<commit_message>
chore: process frontend intake
</commit_message>
<xml_diff>
--- a/reports/dashboard.xlsx
+++ b/reports/dashboard.xlsx
@@ -2069,7 +2069,7 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="N3" s="12" t="inlineStr">
         <is>
-          <t>cruise_intervals</t>
+          <t>operational_smoke</t>
         </is>
       </c>
       <c r="O3" s="12" t="inlineStr">
@@ -2621,12 +2621,12 @@
       </c>
       <c r="AH3" s="12" t="inlineStr">
         <is>
-          <t>Cansada pelo vôlei, mas controlou bem. Aquiles silencioso.</t>
+          <t>Smoke operacional sem commit de resultados. Smoke operacional.</t>
         </is>
       </c>
       <c r="AI3" s="12" t="inlineStr">
         <is>
-          <t>Manter polimento, evitar buscar 5:50/km como treino contínuo.</t>
+          <t>Smoke operacional; nao usar como decisao de treino.</t>
         </is>
       </c>
       <c r="AJ3" s="12" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="AM3" s="12" t="inlineStr">
         <is>
-          <t>["bruna_hr_screenshot","bruna_avg_hr","bruna_max_hr"]</t>
+          <t>["bruna_avg_hr","bruna_max_hr","bruna_hr_screenshot"]</t>
         </is>
       </c>
       <c r="AN3" s="12" t="inlineStr">
@@ -5701,7 +5701,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0</v>
@@ -6180,7 +6180,7 @@
       </c>
       <c r="O3" s="12" t="inlineStr">
         <is>
-          <t>["bruna_hr_screenshot","bruna_avg_hr","bruna_max_hr"]</t>
+          <t>["bruna_avg_hr","bruna_max_hr","bruna_hr_screenshot"]</t>
         </is>
       </c>
       <c r="P3" s="12" t="inlineStr">

</xml_diff>

<commit_message>
fix: harden operational intake safety
</commit_message>
<xml_diff>
--- a/reports/dashboard.xlsx
+++ b/reports/dashboard.xlsx
@@ -1610,11 +1610,9 @@
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>6.17</v>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>6.6</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E18" s="11" t="inlineStr"/>
       <c r="F18" s="11" t="n">
         <v>14.97</v>
       </c>
@@ -1637,9 +1635,11 @@
         </is>
       </c>
       <c r="D19" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="12" t="inlineStr"/>
+        <v>6.17</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>6.6</v>
+      </c>
       <c r="F19" s="12" t="n">
         <v>14.97</v>
       </c>
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>1.33</v>
+        <v>7.47</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>4.37</v>
+        <v>6.78</v>
       </c>
       <c r="F20" s="11" t="n">
         <v>14.97</v>
       </c>
       <c r="G20" s="11" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21">
@@ -1689,16 +1689,16 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>7.47</v>
+        <v>1.33</v>
       </c>
       <c r="E21" s="12" t="n">
-        <v>6.78</v>
+        <v>4.37</v>
       </c>
       <c r="F21" s="12" t="n">
         <v>14.97</v>
       </c>
       <c r="G21" s="12" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2309,17 +2309,17 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>2026-05-28 17:14:17</t>
+          <t>2026-04-13 19:01:28</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -2329,12 +2329,12 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
+          <t>workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
         </is>
       </c>
       <c r="F2" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260528T171417-1p33km-349s-245ee321</t>
+          <t>garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr"/>
@@ -2371,52 +2371,52 @@
       <c r="N2" s="11" t="inlineStr"/>
       <c r="O2" s="11" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>4.02</t>
         </is>
       </c>
       <c r="P2" s="11" t="inlineStr">
         <is>
-          <t>348.7</t>
+          <t>1869.0</t>
         </is>
       </c>
       <c r="Q2" s="11" t="inlineStr">
         <is>
-          <t>4:22</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="R2" s="11" t="inlineStr">
         <is>
-          <t>4:05</t>
+          <t>7:09</t>
         </is>
       </c>
       <c r="S2" s="11" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>142</t>
         </is>
       </c>
       <c r="T2" s="11" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>152</t>
         </is>
       </c>
       <c r="U2" s="11" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>167</t>
         </is>
       </c>
       <c r="V2" s="11" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>216</t>
         </is>
       </c>
       <c r="W2" s="11" t="inlineStr">
         <is>
-          <t>226.0</t>
+          <t>280.0</t>
         </is>
       </c>
       <c r="X2" s="11" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>0.77</t>
         </is>
       </c>
       <c r="Y2" s="11" t="inlineStr"/>
@@ -2468,17 +2468,17 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>2026-05-28 16:17:36</t>
+          <t>2026-04-14 19:08:24</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
@@ -2488,147 +2488,87 @@
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
+          <t>workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260528T161736-7p47km-3039s-17b463bc</t>
+          <t>garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr"/>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>shared_run_with_manual_checkin</t>
+          <t>matheus_garmin_only</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>["matheus","bruna"]</t>
+          <t>["matheus"]</t>
         </is>
       </c>
       <c r="J3" s="12" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="K3" s="12" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>pacer</t>
+          <t>solo</t>
         </is>
       </c>
       <c r="M3" s="12" t="inlineStr">
         <is>
-          <t>Corrida</t>
-        </is>
-      </c>
-      <c r="N3" s="12" t="inlineStr">
-        <is>
-          <t>operational_smoke</t>
-        </is>
-      </c>
+          <t>Treino de força</t>
+        </is>
+      </c>
+      <c r="N3" s="12" t="inlineStr"/>
       <c r="O3" s="12" t="inlineStr">
         <is>
-          <t>7.47</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="P3" s="12" t="inlineStr">
         <is>
-          <t>3039.0</t>
-        </is>
-      </c>
-      <c r="Q3" s="12" t="inlineStr">
-        <is>
-          <t>6:47</t>
-        </is>
-      </c>
-      <c r="R3" s="12" t="inlineStr">
-        <is>
-          <t>4:41</t>
-        </is>
-      </c>
+          <t>22098.0</t>
+        </is>
+      </c>
+      <c r="Q3" s="12" t="inlineStr"/>
+      <c r="R3" s="12" t="inlineStr"/>
       <c r="S3" s="12" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>106</t>
         </is>
       </c>
       <c r="T3" s="12" t="inlineStr">
         <is>
-          <t>164</t>
-        </is>
-      </c>
-      <c r="U3" s="12" t="inlineStr">
-        <is>
-          <t>161</t>
-        </is>
-      </c>
-      <c r="V3" s="12" t="inlineStr">
-        <is>
-          <t>231</t>
-        </is>
-      </c>
-      <c r="W3" s="12" t="inlineStr">
-        <is>
-          <t>264.0</t>
-        </is>
-      </c>
-      <c r="X3" s="12" t="inlineStr">
-        <is>
-          <t>0.91</t>
-        </is>
-      </c>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="U3" s="12" t="inlineStr"/>
+      <c r="V3" s="12" t="inlineStr"/>
+      <c r="W3" s="12" t="inlineStr"/>
+      <c r="X3" s="12" t="inlineStr"/>
       <c r="Y3" s="12" t="inlineStr"/>
       <c r="Z3" s="12" t="inlineStr"/>
-      <c r="AA3" s="12" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
+      <c r="AA3" s="12" t="inlineStr"/>
       <c r="AB3" s="12" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AC3" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AD3" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AE3" s="12" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
-      <c r="AF3" s="12" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="AG3" s="12" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="AH3" s="12" t="inlineStr">
-        <is>
-          <t>Smoke operacional sem commit de resultados. Smoke operacional.</t>
-        </is>
-      </c>
-      <c r="AI3" s="12" t="inlineStr">
-        <is>
-          <t>Smoke operacional; nao usar como decisao de treino.</t>
-        </is>
-      </c>
+      <c r="AC3" s="12" t="inlineStr"/>
+      <c r="AD3" s="12" t="inlineStr"/>
+      <c r="AE3" s="12" t="inlineStr"/>
+      <c r="AF3" s="12" t="inlineStr"/>
+      <c r="AG3" s="12" t="inlineStr"/>
+      <c r="AH3" s="12" t="inlineStr"/>
+      <c r="AI3" s="12" t="inlineStr"/>
       <c r="AJ3" s="12" t="inlineStr">
         <is>
           <t>request_manual_resolution</t>
@@ -2646,7 +2586,7 @@
       </c>
       <c r="AM3" s="12" t="inlineStr">
         <is>
-          <t>["bruna_avg_hr","bruna_max_hr","bruna_hr_screenshot"]</t>
+          <t>["checkin"]</t>
         </is>
       </c>
       <c r="AN3" s="12" t="inlineStr">
@@ -2663,17 +2603,17 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>2026-05-26 17:11:34</t>
+          <t>2026-04-19 18:27:36</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -2683,12 +2623,12 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
+          <t>workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
+          <t>garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr"/>
@@ -2725,52 +2665,52 @@
       <c r="N4" s="11" t="inlineStr"/>
       <c r="O4" s="11" t="inlineStr">
         <is>
-          <t>6.17</t>
+          <t>5.54</t>
         </is>
       </c>
       <c r="P4" s="11" t="inlineStr">
         <is>
-          <t>2445.0</t>
+          <t>2404.0</t>
         </is>
       </c>
       <c r="Q4" s="11" t="inlineStr">
         <is>
-          <t>6:36</t>
+          <t>7:14</t>
         </is>
       </c>
       <c r="R4" s="11" t="inlineStr">
         <is>
-          <t>6:02</t>
+          <t>5:33</t>
         </is>
       </c>
       <c r="S4" s="11" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>148</t>
         </is>
       </c>
       <c r="T4" s="11" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>163</t>
         </is>
       </c>
       <c r="U4" s="11" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>169</t>
         </is>
       </c>
       <c r="V4" s="11" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>228</t>
         </is>
       </c>
       <c r="W4" s="11" t="inlineStr">
         <is>
-          <t>265.0</t>
+          <t>274.0</t>
         </is>
       </c>
       <c r="X4" s="11" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="Y4" s="11" t="inlineStr"/>
@@ -2822,17 +2762,17 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>2026-05-26 00:25:09</t>
+          <t>2026-04-21 12:01:20</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -2842,12 +2782,12 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
+          <t>workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260526T002509-0p00km-6s-63df559b</t>
+          <t>garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr"/>
@@ -2884,30 +2824,54 @@
       <c r="N5" s="12" t="inlineStr"/>
       <c r="O5" s="12" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>6.46</t>
         </is>
       </c>
       <c r="P5" s="12" t="inlineStr">
         <is>
-          <t>5.8</t>
-        </is>
-      </c>
-      <c r="Q5" s="12" t="inlineStr"/>
-      <c r="R5" s="12" t="inlineStr"/>
+          <t>2719.0</t>
+        </is>
+      </c>
+      <c r="Q5" s="12" t="inlineStr">
+        <is>
+          <t>7:01</t>
+        </is>
+      </c>
+      <c r="R5" s="12" t="inlineStr">
+        <is>
+          <t>5:04</t>
+        </is>
+      </c>
       <c r="S5" s="12" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>144</t>
         </is>
       </c>
       <c r="T5" s="12" t="inlineStr">
         <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="U5" s="12" t="inlineStr"/>
-      <c r="V5" s="12" t="inlineStr"/>
-      <c r="W5" s="12" t="inlineStr"/>
-      <c r="X5" s="12" t="inlineStr"/>
+          <t>163</t>
+        </is>
+      </c>
+      <c r="U5" s="12" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="V5" s="12" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="W5" s="12" t="inlineStr">
+        <is>
+          <t>266.0</t>
+        </is>
+      </c>
+      <c r="X5" s="12" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
       <c r="Y5" s="12" t="inlineStr"/>
       <c r="Z5" s="12" t="inlineStr"/>
       <c r="AA5" s="12" t="inlineStr"/>
@@ -2957,17 +2921,17 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>2026-05-24 16:18:30</t>
+          <t>2026-04-25 09:27:55</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -2977,12 +2941,12 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
+          <t>workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260524T161830-5p24km-1833s-5d178a73</t>
+          <t>garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr"/>
@@ -3013,58 +2977,58 @@
       </c>
       <c r="M6" s="11" t="inlineStr">
         <is>
-          <t>Corrida</t>
+          <t>Corrida em esteira</t>
         </is>
       </c>
       <c r="N6" s="11" t="inlineStr"/>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="P6" s="11" t="inlineStr">
         <is>
-          <t>1833.0</t>
+          <t>2112.0</t>
         </is>
       </c>
       <c r="Q6" s="11" t="inlineStr">
         <is>
-          <t>5:50</t>
+          <t>7:20</t>
         </is>
       </c>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>4:54</t>
+          <t>6:55</t>
         </is>
       </c>
       <c r="S6" s="11" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>128</t>
         </is>
       </c>
       <c r="T6" s="11" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>132</t>
         </is>
       </c>
       <c r="U6" s="11" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>169</t>
         </is>
       </c>
       <c r="V6" s="11" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>214</t>
         </is>
       </c>
       <c r="W6" s="11" t="inlineStr">
         <is>
-          <t>258.0</t>
+          <t>275.0</t>
         </is>
       </c>
       <c r="X6" s="11" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="Y6" s="11" t="inlineStr"/>
@@ -3116,17 +3080,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>2026-05-21 15:16:57</t>
+          <t>2026-04-26 18:09:14</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -3136,12 +3100,12 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
+          <t>workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260521T151657-8p85km-3736s-48b5a434</t>
+          <t>garmin-20260426T180914-8p01km-3488s-96e3af94</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr"/>
@@ -3178,52 +3142,52 @@
       <c r="N7" s="12" t="inlineStr"/>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>8.85</t>
+          <t>8.01</t>
         </is>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
-          <t>3736.0</t>
+          <t>3488.0</t>
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr">
         <is>
-          <t>7:02</t>
+          <t>7:15</t>
         </is>
       </c>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>4:07</t>
+          <t>5:35</t>
         </is>
       </c>
       <c r="S7" s="12" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>145</t>
         </is>
       </c>
       <c r="T7" s="12" t="inlineStr">
         <is>
-          <t>185</t>
+          <t>161</t>
         </is>
       </c>
       <c r="U7" s="12" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>169</t>
         </is>
       </c>
       <c r="V7" s="12" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>232</t>
         </is>
       </c>
       <c r="W7" s="12" t="inlineStr">
         <is>
-          <t>268.0</t>
+          <t>273.0</t>
         </is>
       </c>
       <c r="X7" s="12" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="Y7" s="12" t="inlineStr"/>
@@ -3275,17 +3239,17 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>2026-05-18 16:01:25</t>
+          <t>2026-04-28 17:31:06</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -3295,12 +3259,12 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
+          <t>workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
+          <t>garmin-20260428T173106-5p01km-2084s-18eaf306</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr"/>
@@ -3337,52 +3301,52 @@
       <c r="N8" s="11" t="inlineStr"/>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>6.17</t>
+          <t>5.01</t>
         </is>
       </c>
       <c r="P8" s="11" t="inlineStr">
         <is>
-          <t>2426.0</t>
+          <t>2084.0</t>
         </is>
       </c>
       <c r="Q8" s="11" t="inlineStr">
         <is>
-          <t>6:33</t>
+          <t>6:56</t>
         </is>
       </c>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>5:50</t>
+          <t>5:54</t>
         </is>
       </c>
       <c r="S8" s="11" t="inlineStr">
         <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="T8" s="11" t="inlineStr">
+        <is>
           <t>155</t>
         </is>
       </c>
-      <c r="T8" s="11" t="inlineStr">
-        <is>
-          <t>171</t>
-        </is>
-      </c>
       <c r="U8" s="11" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>168</t>
         </is>
       </c>
       <c r="V8" s="11" t="inlineStr">
         <is>
-          <t>248</t>
+          <t>231</t>
         </is>
       </c>
       <c r="W8" s="11" t="inlineStr">
         <is>
-          <t>265.0</t>
+          <t>271.0</t>
         </is>
       </c>
       <c r="X8" s="11" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.85</t>
         </is>
       </c>
       <c r="Y8" s="11" t="inlineStr"/>
@@ -3434,17 +3398,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>2026-05-13 13:15:52</t>
+          <t>2026-05-01 15:58:02</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -3454,12 +3418,12 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
+          <t>workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
+          <t>garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr"/>
@@ -3496,52 +3460,52 @@
       <c r="N9" s="12" t="inlineStr"/>
       <c r="O9" s="12" t="inlineStr">
         <is>
-          <t>7.33</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
-          <t>3049.0</t>
+          <t>2624.0</t>
         </is>
       </c>
       <c r="Q9" s="12" t="inlineStr">
         <is>
-          <t>6:56</t>
+          <t>7:00</t>
         </is>
       </c>
       <c r="R9" s="12" t="inlineStr">
         <is>
-          <t>5:11</t>
+          <t>3:59</t>
         </is>
       </c>
       <c r="S9" s="12" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>160</t>
         </is>
       </c>
       <c r="T9" s="12" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>180</t>
         </is>
       </c>
       <c r="U9" s="12" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>161</t>
         </is>
       </c>
       <c r="V9" s="12" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>230</t>
         </is>
       </c>
       <c r="W9" s="12" t="inlineStr">
         <is>
-          <t>268.0</t>
+          <t>266.0</t>
         </is>
       </c>
       <c r="X9" s="12" t="inlineStr">
         <is>
-          <t>0.92</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="Y9" s="12" t="inlineStr"/>
@@ -3593,17 +3557,17 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10 15:42:38</t>
+          <t>2026-05-03 15:50:18</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -3613,12 +3577,12 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
+          <t>workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
+          <t>garmin-20260503T155018-8p01km-3269s-1ab13585</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr"/>
@@ -3655,42 +3619,42 @@
       <c r="N10" s="11" t="inlineStr"/>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>9.01</t>
+          <t>8.01</t>
         </is>
       </c>
       <c r="P10" s="11" t="inlineStr">
         <is>
-          <t>3581.0</t>
+          <t>3269.0</t>
         </is>
       </c>
       <c r="Q10" s="11" t="inlineStr">
         <is>
-          <t>6:37</t>
+          <t>6:48</t>
         </is>
       </c>
       <c r="R10" s="11" t="inlineStr">
         <is>
-          <t>5:28</t>
+          <t>5:23</t>
         </is>
       </c>
       <c r="S10" s="11" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>145</t>
         </is>
       </c>
       <c r="T10" s="11" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>158</t>
         </is>
       </c>
       <c r="U10" s="11" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>172</t>
         </is>
       </c>
       <c r="V10" s="11" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>246</t>
         </is>
       </c>
       <c r="W10" s="11" t="inlineStr">
@@ -3700,7 +3664,7 @@
       </c>
       <c r="X10" s="11" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.85</t>
         </is>
       </c>
       <c r="Y10" s="11" t="inlineStr"/>
@@ -3752,17 +3716,17 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>2026-05-07 15:40:01</t>
+          <t>2026-05-05 17:52:34</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -3772,12 +3736,12 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
+          <t>workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260507T154001-7p07km-2939s-c562a182</t>
+          <t>garmin-20260505T175234-5p36km-2294s-3884a25e</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr"/>
@@ -3814,52 +3778,52 @@
       <c r="N11" s="12" t="inlineStr"/>
       <c r="O11" s="12" t="inlineStr">
         <is>
-          <t>7.07</t>
+          <t>5.36</t>
         </is>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
-          <t>2939.0</t>
+          <t>2294.0</t>
         </is>
       </c>
       <c r="Q11" s="12" t="inlineStr">
         <is>
-          <t>6:56</t>
+          <t>7:08</t>
         </is>
       </c>
       <c r="R11" s="12" t="inlineStr">
         <is>
-          <t>5:01</t>
+          <t>6:38</t>
         </is>
       </c>
       <c r="S11" s="12" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>149</t>
         </is>
       </c>
       <c r="T11" s="12" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>159</t>
         </is>
       </c>
       <c r="U11" s="12" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>170</t>
         </is>
       </c>
       <c r="V11" s="12" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>225</t>
         </is>
       </c>
       <c r="W11" s="12" t="inlineStr">
         <is>
-          <t>273.0</t>
+          <t>272.0</t>
         </is>
       </c>
       <c r="X11" s="12" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="Y11" s="12" t="inlineStr"/>
@@ -3911,17 +3875,17 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05 17:52:34</t>
+          <t>2026-05-07 15:40:01</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -3931,12 +3895,12 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
+          <t>workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260505T175234-5p36km-2294s-3884a25e</t>
+          <t>garmin-20260507T154001-7p07km-2939s-c562a182</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr"/>
@@ -3973,52 +3937,52 @@
       <c r="N12" s="11" t="inlineStr"/>
       <c r="O12" s="11" t="inlineStr">
         <is>
-          <t>5.36</t>
+          <t>7.07</t>
         </is>
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
-          <t>2294.0</t>
+          <t>2939.0</t>
         </is>
       </c>
       <c r="Q12" s="11" t="inlineStr">
         <is>
-          <t>7:08</t>
+          <t>6:56</t>
         </is>
       </c>
       <c r="R12" s="11" t="inlineStr">
         <is>
-          <t>6:38</t>
+          <t>5:01</t>
         </is>
       </c>
       <c r="S12" s="11" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>145</t>
         </is>
       </c>
       <c r="T12" s="11" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>162</t>
         </is>
       </c>
       <c r="U12" s="11" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>163</t>
         </is>
       </c>
       <c r="V12" s="11" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>237</t>
         </is>
       </c>
       <c r="W12" s="11" t="inlineStr">
         <is>
-          <t>272.0</t>
+          <t>273.0</t>
         </is>
       </c>
       <c r="X12" s="11" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="Y12" s="11" t="inlineStr"/>
@@ -4070,17 +4034,17 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>2026-05-03 15:50:18</t>
+          <t>2026-05-10 15:42:38</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -4090,12 +4054,12 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
+          <t>workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260503T155018-8p01km-3269s-1ab13585</t>
+          <t>garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr"/>
@@ -4132,42 +4096,42 @@
       <c r="N13" s="12" t="inlineStr"/>
       <c r="O13" s="12" t="inlineStr">
         <is>
-          <t>8.01</t>
+          <t>9.01</t>
         </is>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
-          <t>3269.0</t>
+          <t>3581.0</t>
         </is>
       </c>
       <c r="Q13" s="12" t="inlineStr">
         <is>
-          <t>6:48</t>
+          <t>6:37</t>
         </is>
       </c>
       <c r="R13" s="12" t="inlineStr">
         <is>
-          <t>5:23</t>
+          <t>5:28</t>
         </is>
       </c>
       <c r="S13" s="12" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>151</t>
         </is>
       </c>
       <c r="T13" s="12" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>176</t>
         </is>
       </c>
       <c r="U13" s="12" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>171</t>
         </is>
       </c>
       <c r="V13" s="12" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>251</t>
         </is>
       </c>
       <c r="W13" s="12" t="inlineStr">
@@ -4177,7 +4141,7 @@
       </c>
       <c r="X13" s="12" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="Y13" s="12" t="inlineStr"/>
@@ -4229,17 +4193,17 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01 15:58:02</t>
+          <t>2026-05-13 13:15:52</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -4249,12 +4213,12 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
+          <t>workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
+          <t>garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr"/>
@@ -4291,52 +4255,52 @@
       <c r="N14" s="11" t="inlineStr"/>
       <c r="O14" s="11" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>7.33</t>
         </is>
       </c>
       <c r="P14" s="11" t="inlineStr">
         <is>
-          <t>2624.0</t>
+          <t>3049.0</t>
         </is>
       </c>
       <c r="Q14" s="11" t="inlineStr">
         <is>
-          <t>7:00</t>
+          <t>6:56</t>
         </is>
       </c>
       <c r="R14" s="11" t="inlineStr">
         <is>
-          <t>3:59</t>
+          <t>5:11</t>
         </is>
       </c>
       <c r="S14" s="11" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>148</t>
         </is>
       </c>
       <c r="T14" s="11" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>175</t>
         </is>
       </c>
       <c r="U14" s="11" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>156</t>
         </is>
       </c>
       <c r="V14" s="11" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>228</t>
         </is>
       </c>
       <c r="W14" s="11" t="inlineStr">
         <is>
-          <t>266.0</t>
+          <t>268.0</t>
         </is>
       </c>
       <c r="X14" s="11" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="Y14" s="11" t="inlineStr"/>
@@ -4388,17 +4352,17 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>2026-04-28 17:31:06</t>
+          <t>2026-05-18 16:01:25</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -4408,12 +4372,12 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
+          <t>workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260428T173106-5p01km-2084s-18eaf306</t>
+          <t>garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr"/>
@@ -4450,52 +4414,52 @@
       <c r="N15" s="12" t="inlineStr"/>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>5.01</t>
+          <t>6.17</t>
         </is>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
-          <t>2084.0</t>
+          <t>2426.0</t>
         </is>
       </c>
       <c r="Q15" s="12" t="inlineStr">
         <is>
-          <t>6:56</t>
+          <t>6:33</t>
         </is>
       </c>
       <c r="R15" s="12" t="inlineStr">
         <is>
-          <t>5:54</t>
+          <t>5:50</t>
         </is>
       </c>
       <c r="S15" s="12" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>155</t>
         </is>
       </c>
       <c r="T15" s="12" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>171</t>
         </is>
       </c>
       <c r="U15" s="12" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>172</t>
         </is>
       </c>
       <c r="V15" s="12" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>248</t>
         </is>
       </c>
       <c r="W15" s="12" t="inlineStr">
         <is>
-          <t>271.0</t>
+          <t>265.0</t>
         </is>
       </c>
       <c r="X15" s="12" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="Y15" s="12" t="inlineStr"/>
@@ -4547,17 +4511,17 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>2026-04-26 18:09:14</t>
+          <t>2026-05-21 15:16:57</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -4567,12 +4531,12 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
+          <t>workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260426T180914-8p01km-3488s-96e3af94</t>
+          <t>garmin-20260521T151657-8p85km-3736s-48b5a434</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr"/>
@@ -4609,52 +4573,52 @@
       <c r="N16" s="11" t="inlineStr"/>
       <c r="O16" s="11" t="inlineStr">
         <is>
-          <t>8.01</t>
+          <t>8.85</t>
         </is>
       </c>
       <c r="P16" s="11" t="inlineStr">
         <is>
-          <t>3488.0</t>
+          <t>3736.0</t>
         </is>
       </c>
       <c r="Q16" s="11" t="inlineStr">
         <is>
-          <t>7:15</t>
+          <t>7:02</t>
         </is>
       </c>
       <c r="R16" s="11" t="inlineStr">
         <is>
-          <t>5:35</t>
+          <t>4:07</t>
         </is>
       </c>
       <c r="S16" s="11" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>158</t>
         </is>
       </c>
       <c r="T16" s="11" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>185</t>
         </is>
       </c>
       <c r="U16" s="11" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>160</t>
         </is>
       </c>
       <c r="V16" s="11" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>224</t>
         </is>
       </c>
       <c r="W16" s="11" t="inlineStr">
         <is>
-          <t>273.0</t>
+          <t>268.0</t>
         </is>
       </c>
       <c r="X16" s="11" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="Y16" s="11" t="inlineStr"/>
@@ -4706,17 +4670,17 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>2026-04-25 09:27:55</t>
+          <t>2026-05-24 16:18:30</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -4726,12 +4690,12 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
+          <t>workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
+          <t>garmin-20260524T161830-5p24km-1833s-5d178a73</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr"/>
@@ -4762,58 +4726,58 @@
       </c>
       <c r="M17" s="12" t="inlineStr">
         <is>
-          <t>Corrida em esteira</t>
+          <t>Corrida</t>
         </is>
       </c>
       <c r="N17" s="12" t="inlineStr"/>
       <c r="O17" s="12" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.24</t>
         </is>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
-          <t>2112.0</t>
+          <t>1833.0</t>
         </is>
       </c>
       <c r="Q17" s="12" t="inlineStr">
         <is>
-          <t>7:20</t>
+          <t>5:50</t>
         </is>
       </c>
       <c r="R17" s="12" t="inlineStr">
         <is>
-          <t>6:55</t>
+          <t>4:54</t>
         </is>
       </c>
       <c r="S17" s="12" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>162</t>
         </is>
       </c>
       <c r="T17" s="12" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>180</t>
         </is>
       </c>
       <c r="U17" s="12" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>171</t>
         </is>
       </c>
       <c r="V17" s="12" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>287</t>
         </is>
       </c>
       <c r="W17" s="12" t="inlineStr">
         <is>
-          <t>275.0</t>
+          <t>258.0</t>
         </is>
       </c>
       <c r="X17" s="12" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="Y17" s="12" t="inlineStr"/>
@@ -4865,17 +4829,17 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>2026-04-21 12:01:20</t>
+          <t>2026-05-26 00:25:09</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -4885,12 +4849,12 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
+          <t>workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
+          <t>garmin-20260526T002509-0p00km-6s-63df559b</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr"/>
@@ -4927,54 +4891,30 @@
       <c r="N18" s="11" t="inlineStr"/>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>6.46</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="P18" s="11" t="inlineStr">
         <is>
-          <t>2719.0</t>
-        </is>
-      </c>
-      <c r="Q18" s="11" t="inlineStr">
-        <is>
-          <t>7:01</t>
-        </is>
-      </c>
-      <c r="R18" s="11" t="inlineStr">
-        <is>
-          <t>5:04</t>
-        </is>
-      </c>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="Q18" s="11" t="inlineStr"/>
+      <c r="R18" s="11" t="inlineStr"/>
       <c r="S18" s="11" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>80</t>
         </is>
       </c>
       <c r="T18" s="11" t="inlineStr">
         <is>
-          <t>163</t>
-        </is>
-      </c>
-      <c r="U18" s="11" t="inlineStr">
-        <is>
-          <t>161</t>
-        </is>
-      </c>
-      <c r="V18" s="11" t="inlineStr">
-        <is>
-          <t>229</t>
-        </is>
-      </c>
-      <c r="W18" s="11" t="inlineStr">
-        <is>
-          <t>266.0</t>
-        </is>
-      </c>
-      <c r="X18" s="11" t="inlineStr">
-        <is>
-          <t>0.88</t>
-        </is>
-      </c>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="U18" s="11" t="inlineStr"/>
+      <c r="V18" s="11" t="inlineStr"/>
+      <c r="W18" s="11" t="inlineStr"/>
+      <c r="X18" s="11" t="inlineStr"/>
       <c r="Y18" s="11" t="inlineStr"/>
       <c r="Z18" s="11" t="inlineStr"/>
       <c r="AA18" s="11" t="inlineStr"/>
@@ -5024,17 +4964,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>2026-04-19 18:27:36</t>
+          <t>2026-05-26 17:11:34</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -5044,12 +4984,12 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
+          <t>workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
+          <t>garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr"/>
@@ -5086,52 +5026,52 @@
       <c r="N19" s="12" t="inlineStr"/>
       <c r="O19" s="12" t="inlineStr">
         <is>
-          <t>5.54</t>
+          <t>6.17</t>
         </is>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
-          <t>2404.0</t>
+          <t>2445.0</t>
         </is>
       </c>
       <c r="Q19" s="12" t="inlineStr">
         <is>
-          <t>7:14</t>
+          <t>6:36</t>
         </is>
       </c>
       <c r="R19" s="12" t="inlineStr">
         <is>
-          <t>5:33</t>
+          <t>6:02</t>
         </is>
       </c>
       <c r="S19" s="12" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>150</t>
         </is>
       </c>
       <c r="T19" s="12" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>174</t>
         </is>
       </c>
       <c r="U19" s="12" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>171</t>
         </is>
       </c>
       <c r="V19" s="12" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>250</t>
         </is>
       </c>
       <c r="W19" s="12" t="inlineStr">
         <is>
-          <t>274.0</t>
+          <t>265.0</t>
         </is>
       </c>
       <c r="X19" s="12" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="Y19" s="12" t="inlineStr"/>
@@ -5183,17 +5123,17 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>2026-04-14 19:08:24</t>
+          <t>2026-05-28 16:17:36</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -5203,90 +5143,126 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
+          <t>workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
+          <t>garmin-20260528T161736-7p47km-3039s-17b463bc</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr"/>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>matheus_garmin_only</t>
+          <t>shared_run_with_manual_checkin</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>["matheus"]</t>
+          <t>["matheus","bruna"]</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>solo</t>
+          <t>pacer</t>
         </is>
       </c>
       <c r="M20" s="11" t="inlineStr">
         <is>
-          <t>Treino de força</t>
-        </is>
-      </c>
-      <c r="N20" s="11" t="inlineStr"/>
+          <t>Corrida</t>
+        </is>
+      </c>
+      <c r="N20" s="11" t="inlineStr">
+        <is>
+          <t>operational_smoke</t>
+        </is>
+      </c>
       <c r="O20" s="11" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>7.47</t>
         </is>
       </c>
       <c r="P20" s="11" t="inlineStr">
         <is>
-          <t>22098.0</t>
-        </is>
-      </c>
-      <c r="Q20" s="11" t="inlineStr"/>
-      <c r="R20" s="11" t="inlineStr"/>
-      <c r="S20" s="11" t="inlineStr">
-        <is>
-          <t>106</t>
-        </is>
-      </c>
-      <c r="T20" s="11" t="inlineStr">
-        <is>
-          <t>136</t>
-        </is>
-      </c>
+          <t>3039.0</t>
+        </is>
+      </c>
+      <c r="Q20" s="11" t="inlineStr">
+        <is>
+          <t>6:47</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="inlineStr">
+        <is>
+          <t>4:41</t>
+        </is>
+      </c>
+      <c r="S20" s="11" t="inlineStr"/>
+      <c r="T20" s="11" t="inlineStr"/>
       <c r="U20" s="11" t="inlineStr"/>
       <c r="V20" s="11" t="inlineStr"/>
       <c r="W20" s="11" t="inlineStr"/>
       <c r="X20" s="11" t="inlineStr"/>
       <c r="Y20" s="11" t="inlineStr"/>
       <c r="Z20" s="11" t="inlineStr"/>
-      <c r="AA20" s="11" t="inlineStr"/>
+      <c r="AA20" s="11" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="AB20" s="11" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="AC20" s="11" t="inlineStr"/>
-      <c r="AD20" s="11" t="inlineStr"/>
-      <c r="AE20" s="11" t="inlineStr"/>
-      <c r="AF20" s="11" t="inlineStr"/>
-      <c r="AG20" s="11" t="inlineStr"/>
-      <c r="AH20" s="11" t="inlineStr"/>
-      <c r="AI20" s="11" t="inlineStr"/>
+      <c r="AC20" s="11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AD20" s="11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE20" s="11" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="AF20" s="11" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AG20" s="11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AH20" s="11" t="inlineStr">
+        <is>
+          <t>Smoke operacional sem commit de resultados. Smoke operacional.</t>
+        </is>
+      </c>
+      <c r="AI20" s="11" t="inlineStr">
+        <is>
+          <t>Smoke operacional; nao usar como decisao de treino.</t>
+        </is>
+      </c>
       <c r="AJ20" s="11" t="inlineStr">
         <is>
-          <t>request_manual_resolution</t>
+          <t>reduce_next_workout</t>
         </is>
       </c>
       <c r="AK20" s="11" t="inlineStr">
@@ -5301,7 +5277,7 @@
       </c>
       <c r="AM20" s="11" t="inlineStr">
         <is>
-          <t>["checkin"]</t>
+          <t>["bruna_avg_hr","bruna_max_hr","bruna_hr_screenshot"]</t>
         </is>
       </c>
       <c r="AN20" s="11" t="inlineStr">
@@ -5318,17 +5294,17 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>2026-04-13 19:01:28</t>
+          <t>2026-05-28 17:14:17</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -5338,12 +5314,12 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
+          <t>workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
+          <t>garmin-20260528T171417-1p33km-349s-245ee321</t>
         </is>
       </c>
       <c r="G21" s="12" t="inlineStr"/>
@@ -5380,52 +5356,52 @@
       <c r="N21" s="12" t="inlineStr"/>
       <c r="O21" s="12" t="inlineStr">
         <is>
-          <t>4.02</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
-          <t>1869.0</t>
+          <t>348.7</t>
         </is>
       </c>
       <c r="Q21" s="12" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>4:22</t>
         </is>
       </c>
       <c r="R21" s="12" t="inlineStr">
         <is>
-          <t>7:09</t>
+          <t>4:05</t>
         </is>
       </c>
       <c r="S21" s="12" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>189</t>
         </is>
       </c>
       <c r="T21" s="12" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>192</t>
         </is>
       </c>
       <c r="U21" s="12" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>173</t>
         </is>
       </c>
       <c r="V21" s="12" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>357</t>
         </is>
       </c>
       <c r="W21" s="12" t="inlineStr">
         <is>
-          <t>280.0</t>
+          <t>226.0</t>
         </is>
       </c>
       <c r="X21" s="12" t="inlineStr">
         <is>
-          <t>0.77</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="Y21" s="12" t="inlineStr"/>
@@ -5892,7 +5868,7 @@
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
@@ -6008,17 +5984,17 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>2026-05-28 17:14:17</t>
+          <t>2026-04-13 19:01:28</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -6043,12 +6019,12 @@
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
+          <t>workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
@@ -6083,17 +6059,17 @@
       </c>
       <c r="P2" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
+          <t>decision-workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
         </is>
       </c>
       <c r="Q2" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
+          <t>workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
         </is>
       </c>
       <c r="R2" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260528T171417-1p33km-349s-245ee321</t>
+          <t>garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
         </is>
       </c>
       <c r="S2" s="11" t="inlineStr">
@@ -6110,17 +6086,17 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>2026-05-28 16:17:36</t>
+          <t>2026-04-14 19:08:24</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
@@ -6140,22 +6116,22 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Manual check-in matched; recommendation remains deferred until adaptive engine consumes full context.</t>
+          <t>Manual check-in evidence is missing; confidence remains low.</t>
         </is>
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
+          <t>workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
         </is>
       </c>
       <c r="J3" s="12" t="inlineStr">
         <is>
-          <t>manual_checkin</t>
+          <t>garmin_only</t>
         </is>
       </c>
       <c r="K3" s="12" t="inlineStr">
@@ -6180,22 +6156,22 @@
       </c>
       <c r="O3" s="12" t="inlineStr">
         <is>
-          <t>["bruna_avg_hr","bruna_max_hr","bruna_hr_screenshot"]</t>
+          <t>["checkin"]</t>
         </is>
       </c>
       <c r="P3" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
+          <t>decision-workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
         </is>
       </c>
       <c r="Q3" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
+          <t>workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
         </is>
       </c>
       <c r="R3" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260528T161736-7p47km-3039s-17b463bc</t>
+          <t>garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
         </is>
       </c>
       <c r="S3" s="12" t="inlineStr">
@@ -6205,24 +6181,24 @@
       </c>
       <c r="T3" s="12" t="inlineStr">
         <is>
-          <t>Manual check-in matched; recommendation remains deferred until adaptive engine consumes full context.</t>
+          <t>Manual check-in evidence is missing; confidence remains low.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>2026-05-26 17:11:34</t>
+          <t>2026-04-19 18:27:36</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -6247,12 +6223,12 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
+          <t>workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
@@ -6287,17 +6263,17 @@
       </c>
       <c r="P4" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
+          <t>decision-workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
         </is>
       </c>
       <c r="Q4" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
+          <t>workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
         </is>
       </c>
       <c r="R4" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
+          <t>garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
         </is>
       </c>
       <c r="S4" s="11" t="inlineStr">
@@ -6314,17 +6290,17 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>2026-05-26 00:25:09</t>
+          <t>2026-04-21 12:01:20</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -6349,12 +6325,12 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
+          <t>workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
@@ -6389,17 +6365,17 @@
       </c>
       <c r="P5" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
+          <t>decision-workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
+          <t>workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
         </is>
       </c>
       <c r="R5" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260526T002509-0p00km-6s-63df559b</t>
+          <t>garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
         </is>
       </c>
       <c r="S5" s="12" t="inlineStr">
@@ -6416,17 +6392,17 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>2026-05-24 16:18:30</t>
+          <t>2026-04-25 09:27:55</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -6451,12 +6427,12 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
+          <t>workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -6491,17 +6467,17 @@
       </c>
       <c r="P6" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
+          <t>decision-workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
         </is>
       </c>
       <c r="Q6" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
+          <t>workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
         </is>
       </c>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260524T161830-5p24km-1833s-5d178a73</t>
+          <t>garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
         </is>
       </c>
       <c r="S6" s="11" t="inlineStr">
@@ -6518,17 +6494,17 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>2026-05-21 15:16:57</t>
+          <t>2026-04-26 18:09:14</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -6553,12 +6529,12 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
+          <t>workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
@@ -6593,17 +6569,17 @@
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
+          <t>decision-workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
+          <t>workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
         </is>
       </c>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260521T151657-8p85km-3736s-48b5a434</t>
+          <t>garmin-20260426T180914-8p01km-3488s-96e3af94</t>
         </is>
       </c>
       <c r="S7" s="12" t="inlineStr">
@@ -6620,17 +6596,17 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>2026-05-18 16:01:25</t>
+          <t>2026-04-28 17:31:06</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -6655,12 +6631,12 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
+          <t>workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -6695,17 +6671,17 @@
       </c>
       <c r="P8" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
+          <t>decision-workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
         </is>
       </c>
       <c r="Q8" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
+          <t>workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
         </is>
       </c>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
+          <t>garmin-20260428T173106-5p01km-2084s-18eaf306</t>
         </is>
       </c>
       <c r="S8" s="11" t="inlineStr">
@@ -6722,17 +6698,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>2026-05-13 13:15:52</t>
+          <t>2026-05-01 15:58:02</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -6757,12 +6733,12 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
+          <t>workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
@@ -6797,17 +6773,17 @@
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
+          <t>decision-workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
         </is>
       </c>
       <c r="Q9" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
+          <t>workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
         </is>
       </c>
       <c r="R9" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
+          <t>garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
         </is>
       </c>
       <c r="S9" s="12" t="inlineStr">
@@ -6824,17 +6800,17 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10 15:42:38</t>
+          <t>2026-05-03 15:50:18</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -6859,12 +6835,12 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
+          <t>workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
@@ -6899,17 +6875,17 @@
       </c>
       <c r="P10" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
+          <t>decision-workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
         </is>
       </c>
       <c r="Q10" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
+          <t>workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
         </is>
       </c>
       <c r="R10" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
+          <t>garmin-20260503T155018-8p01km-3269s-1ab13585</t>
         </is>
       </c>
       <c r="S10" s="11" t="inlineStr">
@@ -6926,17 +6902,17 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>2026-05-07 15:40:01</t>
+          <t>2026-05-05 17:52:34</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -6961,12 +6937,12 @@
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
+          <t>workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
@@ -7001,17 +6977,17 @@
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
+          <t>decision-workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
         </is>
       </c>
       <c r="Q11" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
+          <t>workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
         </is>
       </c>
       <c r="R11" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260507T154001-7p07km-2939s-c562a182</t>
+          <t>garmin-20260505T175234-5p36km-2294s-3884a25e</t>
         </is>
       </c>
       <c r="S11" s="12" t="inlineStr">
@@ -7028,17 +7004,17 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05 17:52:34</t>
+          <t>2026-05-07 15:40:01</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -7063,12 +7039,12 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
+          <t>workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
@@ -7103,17 +7079,17 @@
       </c>
       <c r="P12" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
+          <t>decision-workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
         </is>
       </c>
       <c r="Q12" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260505T175234-5p36km-2294s-3884a25e</t>
+          <t>workout-garmin-20260507T154001-7p07km-2939s-c562a182</t>
         </is>
       </c>
       <c r="R12" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260505T175234-5p36km-2294s-3884a25e</t>
+          <t>garmin-20260507T154001-7p07km-2939s-c562a182</t>
         </is>
       </c>
       <c r="S12" s="11" t="inlineStr">
@@ -7130,17 +7106,17 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>2026-05-03 15:50:18</t>
+          <t>2026-05-10 15:42:38</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -7165,12 +7141,12 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
+          <t>workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
@@ -7205,17 +7181,17 @@
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
+          <t>decision-workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
         </is>
       </c>
       <c r="Q13" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260503T155018-8p01km-3269s-1ab13585</t>
+          <t>workout-garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
         </is>
       </c>
       <c r="R13" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260503T155018-8p01km-3269s-1ab13585</t>
+          <t>garmin-20260510T154238-9p01km-3581s-04ec4a36</t>
         </is>
       </c>
       <c r="S13" s="12" t="inlineStr">
@@ -7232,17 +7208,17 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>2026-05-01 15:58:02</t>
+          <t>2026-05-13 13:15:52</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -7267,12 +7243,12 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
+          <t>workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
@@ -7307,17 +7283,17 @@
       </c>
       <c r="P14" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
+          <t>decision-workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
         </is>
       </c>
       <c r="Q14" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
+          <t>workout-garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
         </is>
       </c>
       <c r="R14" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260501T155802-6p25km-2624s-031a2d1f</t>
+          <t>garmin-20260513T131552-7p33km-3049s-4f641c6f</t>
         </is>
       </c>
       <c r="S14" s="11" t="inlineStr">
@@ -7334,17 +7310,17 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>2026-04-28 17:31:06</t>
+          <t>2026-05-18 16:01:25</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -7369,12 +7345,12 @@
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
+          <t>workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
@@ -7409,17 +7385,17 @@
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
+          <t>decision-workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
         </is>
       </c>
       <c r="Q15" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260428T173106-5p01km-2084s-18eaf306</t>
+          <t>workout-garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
         </is>
       </c>
       <c r="R15" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260428T173106-5p01km-2084s-18eaf306</t>
+          <t>garmin-20260518T160125-6p17km-2426s-c25e77d9</t>
         </is>
       </c>
       <c r="S15" s="12" t="inlineStr">
@@ -7436,17 +7412,17 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>2026-04-26 18:09:14</t>
+          <t>2026-05-21 15:16:57</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -7471,12 +7447,12 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
+          <t>workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
@@ -7511,17 +7487,17 @@
       </c>
       <c r="P16" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
+          <t>decision-workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
         </is>
       </c>
       <c r="Q16" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260426T180914-8p01km-3488s-96e3af94</t>
+          <t>workout-garmin-20260521T151657-8p85km-3736s-48b5a434</t>
         </is>
       </c>
       <c r="R16" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260426T180914-8p01km-3488s-96e3af94</t>
+          <t>garmin-20260521T151657-8p85km-3736s-48b5a434</t>
         </is>
       </c>
       <c r="S16" s="11" t="inlineStr">
@@ -7538,17 +7514,17 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>2026-04-25 09:27:55</t>
+          <t>2026-05-24 16:18:30</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -7573,12 +7549,12 @@
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
+          <t>workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
@@ -7613,17 +7589,17 @@
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
+          <t>decision-workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
         </is>
       </c>
       <c r="Q17" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
+          <t>workout-garmin-20260524T161830-5p24km-1833s-5d178a73</t>
         </is>
       </c>
       <c r="R17" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260425T092755-4p80km-2112s-e7bdfb0d</t>
+          <t>garmin-20260524T161830-5p24km-1833s-5d178a73</t>
         </is>
       </c>
       <c r="S17" s="12" t="inlineStr">
@@ -7640,17 +7616,17 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>2026-04-21 12:01:20</t>
+          <t>2026-05-26 00:25:09</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -7675,12 +7651,12 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
+          <t>workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
@@ -7715,17 +7691,17 @@
       </c>
       <c r="P18" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
+          <t>decision-workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
         </is>
       </c>
       <c r="Q18" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
+          <t>workout-garmin-20260526T002509-0p00km-6s-63df559b</t>
         </is>
       </c>
       <c r="R18" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260421T120120-6p46km-2719s-a45a4e9b</t>
+          <t>garmin-20260526T002509-0p00km-6s-63df559b</t>
         </is>
       </c>
       <c r="S18" s="11" t="inlineStr">
@@ -7742,17 +7718,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>2026-04-19 18:27:36</t>
+          <t>2026-05-26 17:11:34</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -7777,12 +7753,12 @@
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
+          <t>workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
@@ -7817,17 +7793,17 @@
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
+          <t>decision-workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
         </is>
       </c>
       <c r="Q19" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
+          <t>workout-garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
         </is>
       </c>
       <c r="R19" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260419T182736-5p54km-2404s-ad177ba8</t>
+          <t>garmin-20260526T171134-6p17km-2445s-3da74ec2</t>
         </is>
       </c>
       <c r="S19" s="12" t="inlineStr">
@@ -7844,17 +7820,17 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>2026-04-14 19:08:24</t>
+          <t>2026-05-28 16:17:36</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -7869,42 +7845,42 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>defer</t>
+          <t>reduce</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Manual check-in evidence is missing; confidence remains low.</t>
+          <t>volleyball_previous_day</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: reduce_next_workout.</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
+          <t>workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>garmin_only</t>
+          <t>manual_checkin</t>
         </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["volleyball-neuromuscular-load"]</t>
         </is>
       </c>
       <c r="M20" s="11" t="inlineStr">
         <is>
-          <t>defer</t>
+          <t>reduce</t>
         </is>
       </c>
       <c r="N20" s="11" t="inlineStr">
@@ -7914,49 +7890,49 @@
       </c>
       <c r="O20" s="11" t="inlineStr">
         <is>
-          <t>["checkin"]</t>
+          <t>["bruna_avg_hr","bruna_max_hr","bruna_hr_screenshot"]</t>
         </is>
       </c>
       <c r="P20" s="11" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
+          <t>decision-workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
         </is>
       </c>
       <c r="Q20" s="11" t="inlineStr">
         <is>
-          <t>workout-garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
+          <t>workout-garmin-20260528T161736-7p47km-3039s-17b463bc</t>
         </is>
       </c>
       <c r="R20" s="11" t="inlineStr">
         <is>
-          <t>garmin-20260414T190824-0p00km-22098s-acf0c1f6</t>
+          <t>garmin-20260528T161736-7p47km-3039s-17b463bc</t>
         </is>
       </c>
       <c r="S20" s="11" t="inlineStr">
         <is>
-          <t>request_manual_resolution</t>
+          <t>reduce_next_workout</t>
         </is>
       </c>
       <c r="T20" s="11" t="inlineStr">
         <is>
-          <t>Manual check-in evidence is missing; confidence remains low.</t>
+          <t>volleyball_previous_day</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>2026-04-13 19:01:28</t>
+          <t>2026-05-28 17:14:17</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -7981,12 +7957,12 @@
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>No automatic workout change in Task 7; preserve audit trail for recommendation engine.</t>
+          <t>Deterministic guardrail action: request_manual_resolution.</t>
         </is>
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
+          <t>workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
@@ -8021,17 +7997,17 @@
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
-          <t>decision-workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
+          <t>decision-workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
         </is>
       </c>
       <c r="Q21" s="12" t="inlineStr">
         <is>
-          <t>workout-garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
+          <t>workout-garmin-20260528T171417-1p33km-349s-245ee321</t>
         </is>
       </c>
       <c r="R21" s="12" t="inlineStr">
         <is>
-          <t>garmin-20260413T190128-4p02km-1869s-8dee9c94</t>
+          <t>garmin-20260528T171417-1p33km-349s-245ee321</t>
         </is>
       </c>
       <c r="S21" s="12" t="inlineStr">

</xml_diff>